<commit_message>
Payment integration Phase 1
</commit_message>
<xml_diff>
--- a/docs/OSC_2026-08-30.xlsx
+++ b/docs/OSC_2026-08-30.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{87EBFEBC-3006-4172-A0BC-45871CAFADB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A968B52D-56A4-4963-8FBD-15C2FF853DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{296B55BA-C63C-41FD-A9F1-B8085602E620}"/>
   </bookViews>
   <sheets>
     <sheet name="OSC_2026-08-30" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="337">
   <si>
     <t>shortCode</t>
   </si>
@@ -184,9 +184,6 @@
     <t>DCRTD-NDVDL-CKS</t>
   </si>
   <si>
-    <t>ðŸª</t>
-  </si>
-  <si>
     <t>box cookies</t>
   </si>
   <si>
@@ -202,9 +199,6 @@
     <t>BG-CKS</t>
   </si>
   <si>
-    <t>â˜•ï¸</t>
-  </si>
-  <si>
     <t>Drip coffee</t>
   </si>
   <si>
@@ -229,9 +223,6 @@
     <t>large</t>
   </si>
   <si>
-    <t>ðŸµ</t>
-  </si>
-  <si>
     <t>Tea</t>
   </si>
   <si>
@@ -743,12 +734,6 @@
   </si>
   <si>
     <t>salad</t>
-  </si>
-  <si>
-    <t>Ã— 4 S</t>
-  </si>
-  <si>
-    <t>Ã— 4 Scones</t>
   </si>
   <si>
     <t>Sale Items</t>
@@ -1891,7 +1876,8 @@
   <cols>
     <col min="1" max="1" width="25.28515625" customWidth="1"/>
     <col min="2" max="2" width="39.42578125" customWidth="1"/>
-    <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.85546875" customWidth="1"/>
+    <col min="8" max="8" width="22.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
@@ -2136,14 +2122,11 @@
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>55</v>
-      </c>
-      <c r="C12" t="s">
-        <v>56</v>
       </c>
       <c r="E12">
         <v>10.99</v>
@@ -2154,13 +2137,13 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
         <v>57</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>58</v>
-      </c>
-      <c r="C13" t="s">
-        <v>59</v>
       </c>
       <c r="E13">
         <v>5.99</v>
@@ -2170,14 +2153,11 @@
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" t="s">
         <v>60</v>
-      </c>
-      <c r="B14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" t="s">
-        <v>62</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -2186,42 +2166,39 @@
         <v>26</v>
       </c>
       <c r="G14" t="s">
+        <v>61</v>
+      </c>
+      <c r="H14" t="s">
+        <v>62</v>
+      </c>
+      <c r="I14" t="s">
         <v>63</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>64</v>
-      </c>
-      <c r="I14" t="s">
-        <v>65</v>
-      </c>
-      <c r="J14" t="s">
-        <v>66</v>
       </c>
       <c r="K14">
         <v>2.5</v>
       </c>
       <c r="L14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M14">
         <v>2.8</v>
       </c>
       <c r="N14" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O14">
         <v>3.1</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>69</v>
-      </c>
       <c r="B15" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2230,66 +2207,63 @@
         <v>26</v>
       </c>
       <c r="G15" t="s">
+        <v>61</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" t="s">
         <v>63</v>
       </c>
-      <c r="H15" t="s">
-        <v>72</v>
-      </c>
-      <c r="I15" t="s">
-        <v>65</v>
-      </c>
       <c r="J15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K15">
         <v>2.75</v>
       </c>
       <c r="L15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M15">
         <v>3</v>
       </c>
       <c r="N15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O15">
         <v>3.25</v>
       </c>
       <c r="P15" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="Q15" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="R15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="S15">
         <v>2.75</v>
       </c>
       <c r="T15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="U15">
         <v>3</v>
       </c>
       <c r="V15" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="W15">
         <v>3.25</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>60</v>
-      </c>
       <c r="B16" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2298,42 +2272,39 @@
         <v>26</v>
       </c>
       <c r="G16" t="s">
+        <v>61</v>
+      </c>
+      <c r="H16" t="s">
+        <v>69</v>
+      </c>
+      <c r="I16" t="s">
         <v>63</v>
       </c>
-      <c r="H16" t="s">
-        <v>72</v>
-      </c>
-      <c r="I16" t="s">
-        <v>65</v>
-      </c>
       <c r="J16" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K16">
         <v>3.25</v>
       </c>
       <c r="L16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M16">
         <v>3.5</v>
       </c>
       <c r="N16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O16">
         <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>60</v>
-      </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E17">
         <v>2.1</v>
@@ -2342,18 +2313,15 @@
         <v>26</v>
       </c>
       <c r="G17" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>60</v>
-      </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -2362,42 +2330,39 @@
         <v>26</v>
       </c>
       <c r="G18" t="s">
+        <v>61</v>
+      </c>
+      <c r="H18" t="s">
+        <v>69</v>
+      </c>
+      <c r="I18" t="s">
         <v>63</v>
       </c>
-      <c r="H18" t="s">
-        <v>72</v>
-      </c>
-      <c r="I18" t="s">
-        <v>65</v>
-      </c>
       <c r="J18" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K18">
         <v>3.25</v>
       </c>
       <c r="L18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M18">
         <v>3.75</v>
       </c>
       <c r="N18" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O18">
         <v>4.25</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>60</v>
-      </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -2406,42 +2371,39 @@
         <v>26</v>
       </c>
       <c r="G19" t="s">
+        <v>61</v>
+      </c>
+      <c r="H19" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" t="s">
         <v>63</v>
       </c>
-      <c r="H19" t="s">
-        <v>72</v>
-      </c>
-      <c r="I19" t="s">
-        <v>65</v>
-      </c>
       <c r="J19" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K19">
         <v>3.25</v>
       </c>
       <c r="L19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M19">
         <v>3.75</v>
       </c>
       <c r="N19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O19">
         <v>4.25</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>60</v>
-      </c>
       <c r="B20" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C20" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -2450,42 +2412,39 @@
         <v>26</v>
       </c>
       <c r="G20" t="s">
+        <v>61</v>
+      </c>
+      <c r="H20" t="s">
+        <v>69</v>
+      </c>
+      <c r="I20" t="s">
         <v>63</v>
       </c>
-      <c r="H20" t="s">
-        <v>72</v>
-      </c>
-      <c r="I20" t="s">
-        <v>65</v>
-      </c>
       <c r="J20" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K20">
         <v>4.5</v>
       </c>
       <c r="L20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M20">
         <v>5</v>
       </c>
       <c r="N20" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O20">
         <v>5.5</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>60</v>
-      </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2494,42 +2453,39 @@
         <v>26</v>
       </c>
       <c r="G21" t="s">
+        <v>61</v>
+      </c>
+      <c r="H21" t="s">
+        <v>69</v>
+      </c>
+      <c r="I21" t="s">
         <v>63</v>
       </c>
-      <c r="H21" t="s">
-        <v>72</v>
-      </c>
-      <c r="I21" t="s">
-        <v>65</v>
-      </c>
       <c r="J21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K21">
         <v>3.5</v>
       </c>
       <c r="L21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M21">
         <v>3.89</v>
       </c>
       <c r="N21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O21">
         <v>4.1900000000000004</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>60</v>
-      </c>
       <c r="B22" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2538,42 +2494,39 @@
         <v>26</v>
       </c>
       <c r="G22" t="s">
+        <v>61</v>
+      </c>
+      <c r="H22" t="s">
+        <v>69</v>
+      </c>
+      <c r="I22" t="s">
         <v>63</v>
       </c>
-      <c r="H22" t="s">
-        <v>72</v>
-      </c>
-      <c r="I22" t="s">
-        <v>65</v>
-      </c>
       <c r="J22" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K22">
         <v>3.75</v>
       </c>
       <c r="L22" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M22">
         <v>4.0999999999999996</v>
       </c>
       <c r="N22" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O22">
         <v>4.5</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>60</v>
-      </c>
       <c r="B23" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2582,42 +2535,39 @@
         <v>26</v>
       </c>
       <c r="G23" t="s">
+        <v>61</v>
+      </c>
+      <c r="H23" t="s">
+        <v>69</v>
+      </c>
+      <c r="I23" t="s">
         <v>63</v>
       </c>
-      <c r="H23" t="s">
-        <v>72</v>
-      </c>
-      <c r="I23" t="s">
-        <v>65</v>
-      </c>
       <c r="J23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K23">
         <v>3.25</v>
       </c>
       <c r="L23" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M23">
         <v>3.5</v>
       </c>
       <c r="N23" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O23">
         <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>60</v>
-      </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2626,42 +2576,39 @@
         <v>26</v>
       </c>
       <c r="G24" t="s">
+        <v>61</v>
+      </c>
+      <c r="H24" t="s">
+        <v>69</v>
+      </c>
+      <c r="I24" t="s">
         <v>63</v>
       </c>
-      <c r="H24" t="s">
-        <v>72</v>
-      </c>
-      <c r="I24" t="s">
-        <v>65</v>
-      </c>
       <c r="J24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K24">
         <v>4.0999999999999996</v>
       </c>
       <c r="L24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M24">
         <v>4.6900000000000004</v>
       </c>
       <c r="N24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O24">
         <v>4.99</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>60</v>
-      </c>
       <c r="B25" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2670,42 +2617,39 @@
         <v>26</v>
       </c>
       <c r="G25" t="s">
+        <v>61</v>
+      </c>
+      <c r="H25" t="s">
+        <v>69</v>
+      </c>
+      <c r="I25" t="s">
         <v>63</v>
       </c>
-      <c r="H25" t="s">
-        <v>72</v>
-      </c>
-      <c r="I25" t="s">
-        <v>65</v>
-      </c>
       <c r="J25" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K25">
         <v>3.79</v>
       </c>
       <c r="L25" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M25">
         <v>4</v>
       </c>
       <c r="N25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O25">
         <v>4.29</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>60</v>
-      </c>
       <c r="B26" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2714,42 +2658,39 @@
         <v>26</v>
       </c>
       <c r="G26" t="s">
+        <v>61</v>
+      </c>
+      <c r="H26" t="s">
+        <v>69</v>
+      </c>
+      <c r="I26" t="s">
         <v>63</v>
       </c>
-      <c r="H26" t="s">
-        <v>72</v>
-      </c>
-      <c r="I26" t="s">
-        <v>65</v>
-      </c>
       <c r="J26" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K26">
         <v>4.5</v>
       </c>
       <c r="L26" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M26">
         <v>4.99</v>
       </c>
       <c r="N26" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O26">
         <v>5.49</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>60</v>
-      </c>
       <c r="B27" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C27" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2758,42 +2699,39 @@
         <v>26</v>
       </c>
       <c r="G27" t="s">
+        <v>61</v>
+      </c>
+      <c r="H27" t="s">
+        <v>69</v>
+      </c>
+      <c r="I27" t="s">
         <v>63</v>
       </c>
-      <c r="H27" t="s">
-        <v>72</v>
-      </c>
-      <c r="I27" t="s">
-        <v>65</v>
-      </c>
       <c r="J27" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K27">
         <v>3.75</v>
       </c>
       <c r="L27" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M27">
         <v>4.0999999999999996</v>
       </c>
       <c r="N27" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O27">
         <v>4.5</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>60</v>
-      </c>
       <c r="B28" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C28" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2802,28 +2740,28 @@
         <v>26</v>
       </c>
       <c r="G28" t="s">
+        <v>61</v>
+      </c>
+      <c r="H28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I28" t="s">
         <v>63</v>
       </c>
-      <c r="H28" t="s">
-        <v>72</v>
-      </c>
-      <c r="I28" t="s">
-        <v>65</v>
-      </c>
       <c r="J28" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K28">
         <v>5</v>
       </c>
       <c r="L28" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M28">
         <v>5.45</v>
       </c>
       <c r="N28" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O28">
         <v>5.95</v>
@@ -2831,13 +2769,13 @@
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B29" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E29">
         <v>2.99</v>
@@ -2846,28 +2784,28 @@
         <v>26</v>
       </c>
       <c r="G29" t="s">
+        <v>61</v>
+      </c>
+      <c r="H29" t="s">
+        <v>69</v>
+      </c>
+      <c r="I29" t="s">
         <v>63</v>
       </c>
-      <c r="H29" t="s">
-        <v>72</v>
-      </c>
-      <c r="I29" t="s">
-        <v>65</v>
-      </c>
       <c r="J29" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K29">
         <v>3.3</v>
       </c>
       <c r="L29" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M29">
         <v>3.5</v>
       </c>
       <c r="N29" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O29">
         <v>3.99</v>
@@ -2875,13 +2813,13 @@
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -2890,28 +2828,28 @@
         <v>26</v>
       </c>
       <c r="G30" t="s">
+        <v>61</v>
+      </c>
+      <c r="H30" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" t="s">
         <v>63</v>
       </c>
-      <c r="H30" t="s">
-        <v>72</v>
-      </c>
-      <c r="I30" t="s">
-        <v>65</v>
-      </c>
       <c r="J30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K30">
         <v>3.2</v>
       </c>
       <c r="L30" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M30">
         <v>3.8</v>
       </c>
       <c r="N30" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O30">
         <v>4</v>
@@ -2919,13 +2857,13 @@
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B31" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C31" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E31">
         <v>3.99</v>
@@ -2934,18 +2872,18 @@
         <v>26</v>
       </c>
       <c r="G31" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E32">
         <v>3.99</v>
@@ -2954,18 +2892,18 @@
         <v>26</v>
       </c>
       <c r="G32" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B33" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E33">
         <v>3.99</v>
@@ -2974,18 +2912,18 @@
         <v>26</v>
       </c>
       <c r="G33" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C34" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="E34">
         <v>3.99</v>
@@ -2994,18 +2932,18 @@
         <v>26</v>
       </c>
       <c r="G34" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B35" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C35" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="E35">
         <v>3.99</v>
@@ -3014,18 +2952,18 @@
         <v>26</v>
       </c>
       <c r="G35" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B36" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C36" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E36">
         <v>4.99</v>
@@ -3034,18 +2972,18 @@
         <v>26</v>
       </c>
       <c r="G36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B37" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C37" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="E37">
         <v>3.99</v>
@@ -3054,18 +2992,18 @@
         <v>26</v>
       </c>
       <c r="G37" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B38" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C38" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E38">
         <v>3.99</v>
@@ -3074,18 +3012,18 @@
         <v>26</v>
       </c>
       <c r="G38" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C39" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E39">
         <v>4.99</v>
@@ -3094,18 +3032,18 @@
         <v>26</v>
       </c>
       <c r="G39" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B40" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C40" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="E40">
         <v>4.99</v>
@@ -3114,18 +3052,18 @@
         <v>26</v>
       </c>
       <c r="G40" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B41" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="E41">
         <v>4.99</v>
@@ -3134,18 +3072,18 @@
         <v>26</v>
       </c>
       <c r="G41" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="B42" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C42" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E42">
         <v>3.99</v>
@@ -3154,18 +3092,18 @@
         <v>26</v>
       </c>
       <c r="G42" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B43" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C43" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E43">
         <v>4.99</v>
@@ -3174,18 +3112,18 @@
         <v>26</v>
       </c>
       <c r="G43" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E44">
         <v>4.99</v>
@@ -3194,7 +3132,7 @@
         <v>26</v>
       </c>
       <c r="G44" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
@@ -3214,18 +3152,18 @@
         <v>26</v>
       </c>
       <c r="G45" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B46" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C46" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E46">
         <v>9</v>
@@ -3234,18 +3172,18 @@
         <v>26</v>
       </c>
       <c r="G46" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E47">
         <v>9</v>
@@ -3254,18 +3192,18 @@
         <v>26</v>
       </c>
       <c r="G47" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B48" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C48" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E48">
         <v>3</v>
@@ -3274,18 +3212,18 @@
         <v>26</v>
       </c>
       <c r="G48" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B49" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C49" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="E49">
         <v>5</v>
@@ -3294,18 +3232,18 @@
         <v>26</v>
       </c>
       <c r="G49" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B50" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C50" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="E50">
         <v>3.49</v>
@@ -3314,18 +3252,18 @@
         <v>26</v>
       </c>
       <c r="G50" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B51" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C51" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E51">
         <v>3.49</v>
@@ -3334,18 +3272,18 @@
         <v>26</v>
       </c>
       <c r="G51" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B52" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C52" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="E52">
         <v>3.49</v>
@@ -3354,18 +3292,18 @@
         <v>26</v>
       </c>
       <c r="G52" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B53" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C53" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E53">
         <v>3.49</v>
@@ -3374,18 +3312,18 @@
         <v>26</v>
       </c>
       <c r="G53" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B54" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C54" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E54">
         <v>3.69</v>
@@ -3394,18 +3332,18 @@
         <v>26</v>
       </c>
       <c r="G54" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B55" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C55" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="E55">
         <v>6.5</v>
@@ -3414,18 +3352,18 @@
         <v>26</v>
       </c>
       <c r="G55" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B56" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C56" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="E56">
         <v>1</v>
@@ -3434,18 +3372,18 @@
         <v>26</v>
       </c>
       <c r="G56" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B57" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C57" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="E57">
         <v>6.99</v>
@@ -3454,18 +3392,18 @@
         <v>26</v>
       </c>
       <c r="G57" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B58" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C58" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E58">
         <v>7.99</v>
@@ -3474,18 +3412,18 @@
         <v>26</v>
       </c>
       <c r="G58" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="B59" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C59" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E59">
         <v>6.49</v>
@@ -3494,18 +3432,18 @@
         <v>26</v>
       </c>
       <c r="G59" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B60" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C60" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E60">
         <v>7.99</v>
@@ -3514,18 +3452,18 @@
         <v>26</v>
       </c>
       <c r="G60" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B61" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C61" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E61">
         <v>7.99</v>
@@ -3534,18 +3472,18 @@
         <v>26</v>
       </c>
       <c r="G61" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B62" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C62" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="E62">
         <v>7.99</v>
@@ -3554,18 +3492,18 @@
         <v>26</v>
       </c>
       <c r="G62" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="B63" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C63" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E63">
         <v>7.99</v>
@@ -3574,18 +3512,18 @@
         <v>26</v>
       </c>
       <c r="G63" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B64" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C64" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="E64">
         <v>7.99</v>
@@ -3594,18 +3532,18 @@
         <v>26</v>
       </c>
       <c r="G64" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B65" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C65" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E65">
         <v>8.49</v>
@@ -3614,22 +3552,10 @@
         <v>26</v>
       </c>
       <c r="G65" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A66" t="e">
-        <f>+ GRE</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="B66" t="e">
-        <f>+ greek yogurt</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="C66" t="e">
-        <f>-GRK-YGRT</f>
-        <v>#NAME?</v>
-      </c>
       <c r="E66">
         <v>1</v>
       </c>
@@ -3637,22 +3563,10 @@
         <v>26</v>
       </c>
       <c r="G66" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A67" t="e">
-        <f>+ CHI</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="B67" t="e">
-        <f>+ chia seeds</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="C67" t="e">
-        <f>-CH-SDS</f>
-        <v>#NAME?</v>
-      </c>
       <c r="E67">
         <v>1.1000000000000001</v>
       </c>
@@ -3660,22 +3574,10 @@
         <v>26</v>
       </c>
       <c r="G67" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="e">
-        <f>+ EXT</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="B68" t="e">
-        <f>+ extra fruits</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="C68" t="e">
-        <f>-XTR-FRTS</f>
-        <v>#NAME?</v>
-      </c>
       <c r="E68">
         <v>1</v>
       </c>
@@ -3683,22 +3585,10 @@
         <v>26</v>
       </c>
       <c r="G68" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" t="e">
-        <f>+ OAT</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="B69" t="e">
-        <f>+ OAT milk</f>
-        <v>#NAME?</v>
-      </c>
-      <c r="C69" t="e">
-        <f>-T-MLK</f>
-        <v>#NAME?</v>
-      </c>
       <c r="E69">
         <v>1</v>
       </c>
@@ -3706,18 +3596,18 @@
         <v>26</v>
       </c>
       <c r="G69" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B70" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C70" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="E70">
         <v>1.5</v>
@@ -3726,18 +3616,18 @@
         <v>26</v>
       </c>
       <c r="G70" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B71" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C71" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E71">
         <v>1.5</v>
@@ -3746,18 +3636,18 @@
         <v>26</v>
       </c>
       <c r="G71" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B72" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C72" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E72">
         <v>5.2</v>
@@ -3766,18 +3656,18 @@
         <v>26</v>
       </c>
       <c r="G72" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B73" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C73" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E73">
         <v>3.2</v>
@@ -3786,18 +3676,18 @@
         <v>26</v>
       </c>
       <c r="G73" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B74" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C74" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E74">
         <v>3.2</v>
@@ -3806,18 +3696,18 @@
         <v>26</v>
       </c>
       <c r="G74" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B75" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C75" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="E75">
         <v>8.99</v>
@@ -3826,7 +3716,7 @@
         <v>26</v>
       </c>
       <c r="G75" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
@@ -3834,10 +3724,10 @@
         <v>48</v>
       </c>
       <c r="B76" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C76" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E76">
         <v>7.99</v>
@@ -3846,18 +3736,18 @@
         <v>26</v>
       </c>
       <c r="G76" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B77" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C77" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="E77">
         <v>7.5</v>
@@ -3866,18 +3756,18 @@
         <v>26</v>
       </c>
       <c r="G77" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B78" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C78" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E78">
         <v>6.99</v>
@@ -3886,18 +3776,18 @@
         <v>26</v>
       </c>
       <c r="G78" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B79" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C79" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="E79">
         <v>7.99</v>
@@ -3906,18 +3796,18 @@
         <v>26</v>
       </c>
       <c r="G79" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B80" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C80" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E80">
         <v>7.99</v>
@@ -3926,18 +3816,18 @@
         <v>26</v>
       </c>
       <c r="G80" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="B81" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C81" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E81">
         <v>7.99</v>
@@ -3946,20 +3836,10 @@
         <v>26</v>
       </c>
       <c r="G81" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>241</v>
-      </c>
-      <c r="B82" t="s">
-        <v>242</v>
-      </c>
-      <c r="C82" t="e">
-        <f>-4-SCNS</f>
-        <v>#NAME?</v>
-      </c>
       <c r="E82">
         <v>9</v>
       </c>
@@ -3967,18 +3847,18 @@
         <v>26</v>
       </c>
       <c r="G82" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="B83" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C83" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
       <c r="E83">
         <v>5</v>
@@ -3987,18 +3867,18 @@
         <v>26</v>
       </c>
       <c r="G83" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
       <c r="B84" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
       <c r="C84" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="E84">
         <v>3.99</v>
@@ -4007,18 +3887,18 @@
         <v>26</v>
       </c>
       <c r="G84" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B85" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="C85" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="E85">
         <v>3.99</v>
@@ -4027,18 +3907,18 @@
         <v>26</v>
       </c>
       <c r="G85" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="B86" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="C86" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E86">
         <v>4.6900000000000004</v>
@@ -4047,18 +3927,18 @@
         <v>26</v>
       </c>
       <c r="G86" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="B87" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="C87" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="E87">
         <v>4.99</v>
@@ -4067,18 +3947,18 @@
         <v>26</v>
       </c>
       <c r="G87" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B88" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="C88" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="E88">
         <v>4.99</v>
@@ -4087,18 +3967,18 @@
         <v>26</v>
       </c>
       <c r="G88" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="B89" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="C89" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="E89">
         <v>2.5</v>
@@ -4107,18 +3987,18 @@
         <v>26</v>
       </c>
       <c r="G89" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B90" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C90" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="E90">
         <v>3.99</v>
@@ -4127,18 +4007,18 @@
         <v>26</v>
       </c>
       <c r="G90" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B91" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="C91" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="E91">
         <v>3.99</v>
@@ -4147,18 +4027,18 @@
         <v>26</v>
       </c>
       <c r="G91" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B92" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="C92" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="E92">
         <v>3.99</v>
@@ -4167,18 +4047,18 @@
         <v>26</v>
       </c>
       <c r="G92" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B93" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="C93" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="E93">
         <v>3.99</v>
@@ -4187,18 +4067,18 @@
         <v>26</v>
       </c>
       <c r="G93" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="B94" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="C94" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="E94">
         <v>3.99</v>
@@ -4207,18 +4087,18 @@
         <v>26</v>
       </c>
       <c r="G94" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B95" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C95" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="E95">
         <v>3.99</v>
@@ -4227,18 +4107,18 @@
         <v>26</v>
       </c>
       <c r="G95" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B96" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="C96" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="E96">
         <v>14</v>
@@ -4247,18 +4127,18 @@
         <v>26</v>
       </c>
       <c r="G96" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="B97" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="C97" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="E97">
         <v>1.5</v>
@@ -4267,18 +4147,18 @@
         <v>26</v>
       </c>
       <c r="G97" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B98" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="C98" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="E98">
         <v>2</v>
@@ -4287,18 +4167,18 @@
         <v>26</v>
       </c>
       <c r="G98" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="B99" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="C99" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E99">
         <v>2</v>
@@ -4307,18 +4187,18 @@
         <v>26</v>
       </c>
       <c r="G99" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B100" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="C100" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="E100">
         <v>2</v>
@@ -4327,18 +4207,18 @@
         <v>26</v>
       </c>
       <c r="G100" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B101" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="C101" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="E101">
         <v>2</v>
@@ -4347,18 +4227,18 @@
         <v>26</v>
       </c>
       <c r="G101" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B102" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="C102" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="E102">
         <v>0</v>
@@ -4367,22 +4247,22 @@
         <v>26</v>
       </c>
       <c r="G102" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="H102" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I102" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J102" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="K102">
         <v>6</v>
       </c>
       <c r="L102" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="M102">
         <v>8</v>
@@ -4390,13 +4270,13 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
       <c r="B103" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="C103" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="E103">
         <v>5.2</v>
@@ -4405,18 +4285,18 @@
         <v>26</v>
       </c>
       <c r="G103" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
       <c r="B104" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="C104" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="E104">
         <v>4.8899999999999997</v>
@@ -4425,18 +4305,18 @@
         <v>26</v>
       </c>
       <c r="G104" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="B105" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C105" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="E105">
         <v>4.49</v>
@@ -4445,18 +4325,18 @@
         <v>26</v>
       </c>
       <c r="G105" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="B106" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="C106" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
       <c r="E106">
         <v>4.8899999999999997</v>
@@ -4465,18 +4345,18 @@
         <v>26</v>
       </c>
       <c r="G106" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="B107" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="C107" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="E107">
         <v>4.99</v>
@@ -4485,18 +4365,18 @@
         <v>26</v>
       </c>
       <c r="G107" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
       <c r="B108" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C108" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="E108">
         <v>4.49</v>
@@ -4505,18 +4385,18 @@
         <v>26</v>
       </c>
       <c r="G108" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="B109" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="C109" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="E109">
         <v>12.5</v>
@@ -4525,18 +4405,18 @@
         <v>26</v>
       </c>
       <c r="G109" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="B110" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="C110" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="E110">
         <v>4.49</v>
@@ -4545,7 +4425,7 @@
         <v>26</v>
       </c>
       <c r="G110" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.25">
@@ -4553,10 +4433,10 @@
         <v>27</v>
       </c>
       <c r="B111" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="C111" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="E111">
         <v>4.49</v>
@@ -4565,18 +4445,18 @@
         <v>26</v>
       </c>
       <c r="G111" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B112" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C112" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E112">
         <v>5.49</v>
@@ -4585,18 +4465,18 @@
         <v>26</v>
       </c>
       <c r="G112" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="B113" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="C113" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="E113">
         <v>4.49</v>
@@ -4605,7 +4485,7 @@
         <v>26</v>
       </c>
       <c r="G113" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.25">
@@ -4613,10 +4493,10 @@
         <v>51</v>
       </c>
       <c r="B114" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C114" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="E114">
         <v>6</v>
@@ -4625,18 +4505,18 @@
         <v>26</v>
       </c>
       <c r="G114" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B115" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C115" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="E115">
         <v>9</v>
@@ -4645,18 +4525,18 @@
         <v>26</v>
       </c>
       <c r="G115" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B116" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C116" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E116">
         <v>9</v>
@@ -4665,18 +4545,18 @@
         <v>26</v>
       </c>
       <c r="G116" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>331</v>
+        <v>326</v>
       </c>
       <c r="B117" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="C117" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="E117">
         <v>6.99</v>
@@ -4685,18 +4565,18 @@
         <v>26</v>
       </c>
       <c r="G117" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="B118" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="C118" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="E118">
         <v>7.99</v>
@@ -4705,18 +4585,18 @@
         <v>26</v>
       </c>
       <c r="G118" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="B119" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="C119" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="E119">
         <v>7.49</v>
@@ -4725,7 +4605,7 @@
         <v>26</v>
       </c>
       <c r="G119" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>